<commit_message>
Added command table to serial commands document
</commit_message>
<xml_diff>
--- a/MJ Driver Board/Firmware/Serial commands.xlsx
+++ b/MJ Driver Board/Firmware/Serial commands.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Craig\Documents\GitHub\Xaar128-DW\Products Copy\MJ Driver Board\Firmware\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\patri\GitRepos\AddedScientificDriver\MJ Driver Board\Firmware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6527488B-73B8-4ADE-A765-05635C6DC839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AD5D3DB-84C1-44E0-A0DF-1F5A615576B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Serial commands" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'Serial commands'!$A$1:$E$94</definedName>
+    <definedName name="ExternalData_1" localSheetId="0" hidden="1">'Serial commands'!$A$2:$E$95</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="445" uniqueCount="275">
   <si>
     <t xml:space="preserve">0 </t>
   </si>
@@ -833,6 +833,60 @@
   </si>
   <si>
     <t>Max temperature report function: 71</t>
+  </si>
+  <si>
+    <t>Implemented in Driver Class?</t>
+  </si>
+  <si>
+    <t>Driver.poll_board() - Listener thread updates JSON</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Driver.set_frequency(frequency)</t>
+  </si>
+  <si>
+    <t>Driver.board_reset</t>
+  </si>
+  <si>
+    <t>Driver.activate_nozzles([head_mask], **kwargs) [untested]</t>
+  </si>
+  <si>
+    <t>Driver.check_head_temperatures(). Polls board and returns temperature info from the response data. Currently blocking for 0.2s in calling thread.</t>
+  </si>
+  <si>
+    <t>Driver.set_voltage(head_index, voltage)</t>
+  </si>
+  <si>
+    <t>Driver.clear_heads()</t>
+  </si>
+  <si>
+    <t>Driver.set_encoder_reverse(reverse)</t>
+  </si>
+  <si>
+    <t>Driver.power_off()</t>
+  </si>
+  <si>
+    <t>Driver.fill_head(head_index)</t>
+  </si>
+  <si>
+    <t>Driver.set_mode(mode). Mode is setup as an enum type in Driver Class</t>
+  </si>
+  <si>
+    <t>Driver.activate_nozzle_span(head_index, start_nozzle, span_length)</t>
+  </si>
+  <si>
+    <t>Driver.power_on()</t>
+  </si>
+  <si>
+    <t>Driver.stop_head_heating()</t>
+  </si>
+  <si>
+    <t>Driver.set_head_temperature(head_index,  temperature)</t>
+  </si>
+  <si>
+    <t>Driver.set_start_position(start_position)</t>
   </si>
 </sst>
 </file>
@@ -1321,14 +1375,20 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1375,7 +1435,10 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="6">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1406,8 +1469,8 @@
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" connectionId="2" xr16:uid="{00000000-0016-0000-0000-000000000000}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
-  <queryTableRefresh nextId="9" unboundColumnsRight="2">
-    <queryTableFields count="7">
+  <queryTableRefresh nextId="10" unboundColumnsRight="3">
+    <queryTableFields count="8">
       <queryTableField id="1" name="Column1" tableColumnId="1"/>
       <queryTableField id="2" name="Column2" tableColumnId="2"/>
       <queryTableField id="5" dataBound="0" tableColumnId="5"/>
@@ -1415,14 +1478,15 @@
       <queryTableField id="3" name="Column3" tableColumnId="3"/>
       <queryTableField id="7" dataBound="0" tableColumnId="7"/>
       <queryTableField id="8" dataBound="0" tableColumnId="8"/>
+      <queryTableField id="9" dataBound="0" tableColumnId="9"/>
     </queryTableFields>
   </queryTableRefresh>
 </queryTable>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Serial_commands__2" displayName="Serial_commands__2" ref="A1:G94" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:G94" xr:uid="{00000000-0009-0000-0100-000002000000}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Serial_commands__2" displayName="Serial_commands__2" ref="A2:H95" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A2:H95" xr:uid="{00000000-0009-0000-0100-000002000000}">
     <filterColumn colId="1">
       <filters>
         <filter val="A command to immediately turn off head heating."/>
@@ -1460,23 +1524,24 @@
       </filters>
     </filterColumn>
   </autoFilter>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" uniqueName="1" name="Char" queryTableFieldId="1" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" uniqueName="2" name="Command" queryTableFieldId="2" dataDxfId="3"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" uniqueName="1" name="Char" queryTableFieldId="1" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" uniqueName="2" name="Command" queryTableFieldId="2" dataDxfId="4"/>
     <tableColumn id="5" xr3:uid="{F02E788B-ABAC-D84D-BCAD-F4555D9250E9}" uniqueName="5" name="Category" queryTableFieldId="5"/>
     <tableColumn id="4" xr3:uid="{C3A18F71-AEB6-A64F-8F57-DA18A63AE603}" uniqueName="4" name="Description" queryTableFieldId="4"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" uniqueName="3" name="Arguments" queryTableFieldId="3" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{D8B1A7DB-AD8E-440E-AAA0-82F4E675F00A}" uniqueName="7" name="Example (+&quot;LF&quot;)" queryTableFieldId="7" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{72251A22-B00C-400B-8EBC-DC2DA4FD6EBC}" uniqueName="8" name="Response" queryTableFieldId="8" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" uniqueName="3" name="Arguments" queryTableFieldId="3" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{D8B1A7DB-AD8E-440E-AAA0-82F4E675F00A}" uniqueName="7" name="Example (+&quot;LF&quot;)" queryTableFieldId="7" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{72251A22-B00C-400B-8EBC-DC2DA4FD6EBC}" uniqueName="8" name="Response" queryTableFieldId="8" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{744B75F8-4200-4C40-BFB9-C7C45B7432FB}" uniqueName="9" name="Implemented in Driver Class?" queryTableFieldId="9" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1514,7 +1579,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1620,7 +1685,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1762,7 +1827,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1770,1567 +1835,1605 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G94"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <dimension ref="A2:H95"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="7.140625" customWidth="1"/>
-    <col min="2" max="2" width="59.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="59.42578125" customWidth="1"/>
-    <col min="4" max="4" width="13.28515625" customWidth="1"/>
-    <col min="5" max="5" width="45.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="45.28515625" customWidth="1"/>
+    <col min="1" max="1" width="7.109375" customWidth="1"/>
+    <col min="2" max="2" width="59.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="45.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="45.33203125" customWidth="1"/>
+    <col min="8" max="8" width="27.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" t="s">
+    <row r="2" spans="1:8">
+      <c r="A2" t="s">
         <v>139</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
         <v>140</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C2" t="s">
         <v>145</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D2" t="s">
         <v>142</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E2" t="s">
         <v>141</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F2" t="s">
         <v>192</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G2" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" hidden="1">
-      <c r="A2" t="s">
+      <c r="H2" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" hidden="1">
+      <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-    </row>
-    <row r="3" spans="1:7" hidden="1">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" spans="1:8" hidden="1">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
-      <c r="E3" t="s">
-        <v>2</v>
-      </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-    </row>
-    <row r="4" spans="1:7" hidden="1">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" spans="1:8" hidden="1">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
-        <v>1</v>
-      </c>
-      <c r="E4" t="s">
-        <v>2</v>
-      </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-    </row>
-    <row r="5" spans="1:7" hidden="1">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" t="s">
+        <v>2</v>
+      </c>
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6" spans="1:8" hidden="1">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B5" t="s">
-        <v>1</v>
-      </c>
-      <c r="E5" t="s">
-        <v>2</v>
-      </c>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-    </row>
-    <row r="6" spans="1:7" hidden="1">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H6" s="3"/>
+    </row>
+    <row r="7" spans="1:8" hidden="1">
+      <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6" t="s">
-        <v>2</v>
-      </c>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-    </row>
-    <row r="7" spans="1:7" hidden="1">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E7" t="s">
+        <v>2</v>
+      </c>
+      <c r="H7" s="3"/>
+    </row>
+    <row r="8" spans="1:8" hidden="1">
+      <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B7" t="s">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
-        <v>2</v>
-      </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-    </row>
-    <row r="8" spans="1:7" hidden="1">
-      <c r="A8" t="s">
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>2</v>
+      </c>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" spans="1:8" hidden="1">
+      <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B8" t="s">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>2</v>
-      </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-    </row>
-    <row r="9" spans="1:7" hidden="1">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" t="s">
+        <v>2</v>
+      </c>
+      <c r="H9" s="3"/>
+    </row>
+    <row r="10" spans="1:8" hidden="1">
+      <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B9" t="s">
-        <v>1</v>
-      </c>
-      <c r="E9" t="s">
-        <v>2</v>
-      </c>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:7" hidden="1">
-      <c r="A10" t="s">
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>2</v>
+      </c>
+      <c r="H10" s="3"/>
+    </row>
+    <row r="11" spans="1:8" hidden="1">
+      <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B10" t="s">
-        <v>1</v>
-      </c>
-      <c r="E10" t="s">
-        <v>2</v>
-      </c>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-    </row>
-    <row r="11" spans="1:7" hidden="1">
-      <c r="A11" t="s">
+      <c r="B11" t="s">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
+        <v>2</v>
+      </c>
+      <c r="H11" s="3"/>
+    </row>
+    <row r="12" spans="1:8" hidden="1">
+      <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="B11" t="s">
-        <v>1</v>
-      </c>
-      <c r="E11" t="s">
-        <v>2</v>
-      </c>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-    </row>
-    <row r="12" spans="1:7" hidden="1">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
+        <v>1</v>
+      </c>
+      <c r="E12" t="s">
+        <v>2</v>
+      </c>
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" spans="1:8" hidden="1">
+      <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B12" t="s">
-        <v>1</v>
-      </c>
-      <c r="E12" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-    </row>
-    <row r="13" spans="1:7" ht="409.5">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
       <c r="B13" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D13" t="s">
-        <v>143</v>
+        <v>1</v>
       </c>
       <c r="E13" t="s">
         <v>13</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" hidden="1">
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" spans="1:8" ht="409.6">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
-        <v>1</v>
+        <v>15</v>
+      </c>
+      <c r="C14" t="s">
+        <v>146</v>
+      </c>
+      <c r="D14" t="s">
+        <v>143</v>
       </c>
       <c r="E14" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="1"/>
+      <c r="F14" t="s">
+        <v>193</v>
+      </c>
       <c r="G14" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" hidden="1">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E15" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="1" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" hidden="1">
-      <c r="A15" t="s">
+      <c r="H15" s="5"/>
+    </row>
+    <row r="16" spans="1:8" hidden="1">
+      <c r="A16" t="s">
         <v>17</v>
       </c>
-      <c r="B15" t="s">
-        <v>1</v>
-      </c>
-      <c r="E15" t="s">
-        <v>2</v>
-      </c>
-      <c r="F15" s="1"/>
-      <c r="G15" s="2" t="s">
+      <c r="B16" t="s">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
+        <v>2</v>
+      </c>
+      <c r="G16" s="1" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" hidden="1">
-      <c r="A16" t="s">
+      <c r="H16" s="5"/>
+    </row>
+    <row r="17" spans="1:8" hidden="1">
+      <c r="A17" t="s">
         <v>18</v>
       </c>
-      <c r="B16" t="s">
-        <v>1</v>
-      </c>
-      <c r="E16" t="s">
+      <c r="B17" t="s">
+        <v>1</v>
+      </c>
+      <c r="E17" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-    </row>
-    <row r="17" spans="1:7" hidden="1">
-      <c r="A17" t="s">
+      <c r="H17" s="3"/>
+    </row>
+    <row r="18" spans="1:8" hidden="1">
+      <c r="A18" t="s">
         <v>20</v>
       </c>
-      <c r="B17" t="s">
-        <v>1</v>
-      </c>
-      <c r="E17" t="s">
-        <v>2</v>
-      </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-    </row>
-    <row r="18" spans="1:7" hidden="1">
-      <c r="A18" t="s">
+      <c r="B18" t="s">
+        <v>1</v>
+      </c>
+      <c r="E18" t="s">
+        <v>2</v>
+      </c>
+      <c r="H18" s="3"/>
+    </row>
+    <row r="19" spans="1:8" hidden="1">
+      <c r="A19" t="s">
         <v>21</v>
       </c>
-      <c r="B18" t="s">
-        <v>1</v>
-      </c>
-      <c r="E18" t="s">
-        <v>2</v>
-      </c>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-    </row>
-    <row r="19" spans="1:7" hidden="1">
-      <c r="A19" t="s">
+      <c r="B19" t="s">
+        <v>1</v>
+      </c>
+      <c r="E19" t="s">
+        <v>2</v>
+      </c>
+      <c r="H19" s="3"/>
+    </row>
+    <row r="20" spans="1:8" hidden="1">
+      <c r="A20" t="s">
         <v>22</v>
       </c>
-      <c r="B19" t="s">
-        <v>1</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="B20" t="s">
+        <v>1</v>
+      </c>
+      <c r="E20" t="s">
         <v>13</v>
       </c>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-    </row>
-    <row r="20" spans="1:7" hidden="1">
-      <c r="A20" t="s">
+      <c r="H20" s="3"/>
+    </row>
+    <row r="21" spans="1:8" hidden="1">
+      <c r="A21" t="s">
         <v>23</v>
       </c>
-      <c r="B20" t="s">
-        <v>1</v>
-      </c>
-      <c r="E20" t="s">
-        <v>2</v>
-      </c>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-    </row>
-    <row r="21" spans="1:7" hidden="1">
-      <c r="A21" t="s">
+      <c r="B21" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21" t="s">
+        <v>2</v>
+      </c>
+      <c r="H21" s="3"/>
+    </row>
+    <row r="22" spans="1:8" hidden="1">
+      <c r="A22" t="s">
         <v>24</v>
       </c>
-      <c r="B21" t="s">
-        <v>1</v>
-      </c>
-      <c r="E21" t="s">
-        <v>2</v>
-      </c>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
+        <v>1</v>
+      </c>
+      <c r="E22" t="s">
+        <v>2</v>
+      </c>
+      <c r="H22" s="3"/>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
         <v>25</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B23" t="s">
         <v>26</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C23" t="s">
         <v>148</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D23" t="s">
         <v>144</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E23" t="s">
         <v>13</v>
       </c>
-      <c r="F22" s="1" t="s">
+      <c r="F23" t="s">
         <v>198</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="G23" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" hidden="1">
-      <c r="A23" t="s">
+      <c r="H23" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" hidden="1">
+      <c r="A24" t="s">
         <v>27</v>
       </c>
-      <c r="B23" t="s">
-        <v>1</v>
-      </c>
-      <c r="E23" t="s">
-        <v>2</v>
-      </c>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-    </row>
-    <row r="24" spans="1:7" hidden="1">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
+        <v>1</v>
+      </c>
+      <c r="E24" t="s">
+        <v>2</v>
+      </c>
+      <c r="H24" s="3"/>
+    </row>
+    <row r="25" spans="1:8" hidden="1">
+      <c r="A25" t="s">
         <v>28</v>
       </c>
-      <c r="B24" t="s">
-        <v>1</v>
-      </c>
-      <c r="E24" t="s">
+      <c r="B25" t="s">
+        <v>1</v>
+      </c>
+      <c r="E25" t="s">
         <v>29</v>
       </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" t="s">
+      <c r="H25" s="3"/>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" t="s">
         <v>30</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B26" t="s">
         <v>31</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C26" t="s">
         <v>149</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D26" t="s">
         <v>169</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E26" t="s">
         <v>32</v>
       </c>
-      <c r="F25" s="1" t="s">
+      <c r="F26" t="s">
         <v>204</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="G26" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" hidden="1">
-      <c r="A26" t="s">
+      <c r="H26" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" hidden="1">
+      <c r="A27" t="s">
         <v>33</v>
       </c>
-      <c r="B26" t="s">
-        <v>1</v>
-      </c>
-      <c r="E26" t="s">
-        <v>2</v>
-      </c>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-    </row>
-    <row r="27" spans="1:7" ht="30">
-      <c r="A27" t="s">
+      <c r="B27" t="s">
+        <v>1</v>
+      </c>
+      <c r="E27" t="s">
+        <v>2</v>
+      </c>
+      <c r="H27" s="3"/>
+    </row>
+    <row r="28" spans="1:8" ht="28.8">
+      <c r="A28" t="s">
         <v>34</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B28" t="s">
         <v>35</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C28" t="s">
         <v>150</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D28" t="s">
         <v>151</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E28" t="s">
         <v>36</v>
       </c>
-      <c r="F27" s="1" t="s">
+      <c r="F28" t="s">
         <v>206</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G28" s="2" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="A28" t="s">
+      <c r="H28" s="4" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" t="s">
         <v>37</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B29" t="s">
         <v>38</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C29" t="s">
         <v>148</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D29" t="s">
         <v>152</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E29" t="s">
         <v>39</v>
       </c>
-      <c r="F28" s="1" t="s">
+      <c r="F29" t="s">
         <v>208</v>
       </c>
-      <c r="G28" s="1" t="s">
+      <c r="G29" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" ht="30">
-      <c r="A29" t="s">
+      <c r="H29" s="3"/>
+    </row>
+    <row r="30" spans="1:8" ht="28.8">
+      <c r="A30" t="s">
         <v>40</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B30" t="s">
         <v>41</v>
-      </c>
-      <c r="C29" t="s">
-        <v>150</v>
-      </c>
-      <c r="D29" t="s">
-        <v>170</v>
-      </c>
-      <c r="E29" t="s">
-        <v>13</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="G29" s="3" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="A30" t="s">
-        <v>42</v>
-      </c>
-      <c r="B30" t="s">
-        <v>215</v>
       </c>
       <c r="C30" t="s">
         <v>150</v>
       </c>
       <c r="D30" t="s">
+        <v>170</v>
+      </c>
+      <c r="E30" t="s">
+        <v>13</v>
+      </c>
+      <c r="F30" t="s">
+        <v>199</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" t="s">
+        <v>215</v>
+      </c>
+      <c r="C31" t="s">
+        <v>150</v>
+      </c>
+      <c r="D31" t="s">
         <v>216</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E31" t="s">
         <v>219</v>
       </c>
-      <c r="F30" s="1" t="s">
+      <c r="F31" t="s">
         <v>217</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="G31" t="s">
         <v>218</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" ht="75">
-      <c r="A31" t="s">
+      <c r="H31" s="3" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="86.4">
+      <c r="A32" t="s">
         <v>43</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>44</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C32" t="s">
         <v>146</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D32" t="s">
         <v>153</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E32" t="s">
         <v>13</v>
       </c>
-      <c r="F31" s="1" t="s">
+      <c r="F32" t="s">
         <v>200</v>
       </c>
-      <c r="G31" s="3" t="s">
+      <c r="G32" s="2" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" hidden="1">
-      <c r="A32" t="s">
+      <c r="H32" s="4" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" hidden="1">
+      <c r="A33" t="s">
         <v>45</v>
       </c>
-      <c r="B32" t="s">
-        <v>1</v>
-      </c>
-      <c r="E32" t="s">
-        <v>2</v>
-      </c>
-      <c r="F32" s="1"/>
-      <c r="G32" s="1"/>
-    </row>
-    <row r="33" spans="1:7">
-      <c r="A33" t="s">
+      <c r="B33" t="s">
+        <v>1</v>
+      </c>
+      <c r="E33" t="s">
+        <v>2</v>
+      </c>
+      <c r="H33" s="3"/>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" t="s">
         <v>46</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B34" t="s">
         <v>47</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C34" t="s">
         <v>147</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D34" t="s">
         <v>171</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E34" t="s">
         <v>48</v>
       </c>
-      <c r="F33" s="1" t="s">
+      <c r="F34" t="s">
         <v>225</v>
       </c>
-      <c r="G33" s="1" t="s">
+      <c r="G34" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" hidden="1">
-      <c r="A34" t="s">
+      <c r="H34" s="3" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" hidden="1">
+      <c r="A35" t="s">
         <v>49</v>
       </c>
-      <c r="B34" t="s">
-        <v>1</v>
-      </c>
-      <c r="E34" t="s">
-        <v>2</v>
-      </c>
-      <c r="F34" s="1"/>
-      <c r="G34" s="1"/>
-    </row>
-    <row r="35" spans="1:7" hidden="1">
-      <c r="A35" t="s">
+      <c r="B35" t="s">
+        <v>1</v>
+      </c>
+      <c r="E35" t="s">
+        <v>2</v>
+      </c>
+      <c r="H35" s="3"/>
+    </row>
+    <row r="36" spans="1:8" hidden="1">
+      <c r="A36" t="s">
         <v>50</v>
       </c>
-      <c r="B35" t="s">
-        <v>1</v>
-      </c>
-      <c r="E35" t="s">
-        <v>2</v>
-      </c>
-      <c r="F35" s="1"/>
-      <c r="G35" s="1"/>
-    </row>
-    <row r="36" spans="1:7" hidden="1">
-      <c r="A36" t="s">
+      <c r="B36" t="s">
+        <v>1</v>
+      </c>
+      <c r="E36" t="s">
+        <v>2</v>
+      </c>
+      <c r="H36" s="3"/>
+    </row>
+    <row r="37" spans="1:8" hidden="1">
+      <c r="A37" t="s">
         <v>51</v>
       </c>
-      <c r="B36" t="s">
-        <v>1</v>
-      </c>
-      <c r="E36" t="s">
-        <v>2</v>
-      </c>
-      <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
-    </row>
-    <row r="37" spans="1:7" hidden="1">
-      <c r="A37" t="s">
+      <c r="B37" t="s">
+        <v>1</v>
+      </c>
+      <c r="E37" t="s">
+        <v>2</v>
+      </c>
+      <c r="H37" s="3"/>
+    </row>
+    <row r="38" spans="1:8" hidden="1">
+      <c r="A38" t="s">
         <v>52</v>
       </c>
-      <c r="B37" t="s">
-        <v>1</v>
-      </c>
-      <c r="E37" t="s">
-        <v>2</v>
-      </c>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-    </row>
-    <row r="38" spans="1:7" ht="60">
-      <c r="A38" t="s">
+      <c r="B38" t="s">
+        <v>1</v>
+      </c>
+      <c r="E38" t="s">
+        <v>2</v>
+      </c>
+      <c r="H38" s="3"/>
+    </row>
+    <row r="39" spans="1:8" ht="57.6">
+      <c r="A39" t="s">
         <v>53</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B39" t="s">
         <v>54</v>
-      </c>
-      <c r="C38" t="s">
-        <v>146</v>
-      </c>
-      <c r="D38" t="s">
-        <v>172</v>
-      </c>
-      <c r="E38" t="s">
-        <v>55</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="30">
-      <c r="A39" t="s">
-        <v>56</v>
-      </c>
-      <c r="B39" t="s">
-        <v>57</v>
       </c>
       <c r="C39" t="s">
         <v>146</v>
       </c>
       <c r="D39" t="s">
+        <v>172</v>
+      </c>
+      <c r="E39" t="s">
+        <v>55</v>
+      </c>
+      <c r="F39" t="s">
+        <v>209</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="28.8">
+      <c r="A40" t="s">
+        <v>56</v>
+      </c>
+      <c r="B40" t="s">
+        <v>57</v>
+      </c>
+      <c r="C40" t="s">
+        <v>146</v>
+      </c>
+      <c r="D40" t="s">
         <v>154</v>
       </c>
-      <c r="E39" t="s">
+      <c r="E40" t="s">
         <v>58</v>
       </c>
-      <c r="F39" s="1" t="s">
+      <c r="F40" t="s">
         <v>201</v>
       </c>
-      <c r="G39" s="3" t="s">
+      <c r="G40" s="2" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="40" spans="1:7">
-      <c r="A40" t="s">
+      <c r="H40" s="4" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" t="s">
         <v>59</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>60</v>
       </c>
-      <c r="C40" t="s">
+      <c r="C41" t="s">
         <v>149</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D41" t="s">
         <v>155</v>
       </c>
-      <c r="E40" t="s">
+      <c r="E41" t="s">
         <v>13</v>
       </c>
-      <c r="F40" s="1" t="s">
+      <c r="F41" t="s">
         <v>202</v>
       </c>
-      <c r="G40" s="1" t="s">
+      <c r="G41" t="s">
         <v>230</v>
       </c>
-    </row>
-    <row r="41" spans="1:7">
-      <c r="A41" t="s">
+      <c r="H41" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" t="s">
         <v>61</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B42" t="s">
         <v>62</v>
       </c>
-      <c r="C41" t="s">
+      <c r="C42" t="s">
         <v>148</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D42" t="s">
         <v>156</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E42" t="s">
         <v>63</v>
       </c>
-      <c r="F41" s="1" t="s">
+      <c r="F42" t="s">
         <v>210</v>
       </c>
-      <c r="G41" s="1" t="s">
+      <c r="G42" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" hidden="1">
-      <c r="A42" t="s">
+      <c r="H42" s="3" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" hidden="1">
+      <c r="A43" t="s">
         <v>64</v>
       </c>
-      <c r="B42" t="s">
-        <v>1</v>
-      </c>
-      <c r="E42" t="s">
-        <v>13</v>
-      </c>
-      <c r="F42" s="1"/>
-      <c r="G42" s="1"/>
-    </row>
-    <row r="43" spans="1:7">
-      <c r="A43" t="s">
-        <v>65</v>
-      </c>
       <c r="B43" t="s">
-        <v>66</v>
-      </c>
-      <c r="C43" t="s">
-        <v>150</v>
-      </c>
-      <c r="D43" t="s">
-        <v>157</v>
+        <v>1</v>
       </c>
       <c r="E43" t="s">
         <v>13</v>
       </c>
-      <c r="F43" s="1" t="s">
+      <c r="H43" s="3"/>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" t="s">
+        <v>65</v>
+      </c>
+      <c r="B44" t="s">
+        <v>66</v>
+      </c>
+      <c r="C44" t="s">
+        <v>150</v>
+      </c>
+      <c r="D44" t="s">
+        <v>157</v>
+      </c>
+      <c r="E44" t="s">
+        <v>13</v>
+      </c>
+      <c r="F44" t="s">
         <v>203</v>
       </c>
-      <c r="G43" s="1" t="s">
+      <c r="G44" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="44" spans="1:7">
-      <c r="A44" t="s">
+      <c r="H44" s="3" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" t="s">
         <v>67</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B45" t="s">
         <v>68</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C45" t="s">
         <v>147</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D45" t="s">
         <v>158</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E45" t="s">
         <v>69</v>
       </c>
-      <c r="F44" s="1" t="s">
+      <c r="F45" t="s">
         <v>233</v>
       </c>
-      <c r="G44" s="1">
+      <c r="G45">
         <v>1000000</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" hidden="1">
-      <c r="A45" t="s">
+      <c r="H45" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" hidden="1">
+      <c r="A46" t="s">
         <v>70</v>
       </c>
-      <c r="B45" t="s">
-        <v>1</v>
-      </c>
-      <c r="E45" t="s">
-        <v>2</v>
-      </c>
-      <c r="F45" s="1"/>
-      <c r="G45" s="1"/>
-    </row>
-    <row r="46" spans="1:7">
-      <c r="A46" t="s">
+      <c r="B46" t="s">
+        <v>1</v>
+      </c>
+      <c r="E46" t="s">
+        <v>2</v>
+      </c>
+      <c r="H46" s="3"/>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" t="s">
         <v>71</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B47" t="s">
         <v>72</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C47" t="s">
         <v>149</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D47" t="s">
         <v>173</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E47" t="s">
         <v>73</v>
       </c>
-      <c r="F46" s="1" t="s">
+      <c r="F47" t="s">
         <v>211</v>
       </c>
-      <c r="G46" s="1" t="s">
+      <c r="G47" t="s">
         <v>234</v>
       </c>
-    </row>
-    <row r="47" spans="1:7">
-      <c r="A47" t="s">
+      <c r="H47" s="3" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
+      <c r="A48" t="s">
         <v>74</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B48" t="s">
         <v>162</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C48" t="s">
         <v>164</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D48" t="s">
         <v>174</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E48" t="s">
         <v>165</v>
       </c>
-      <c r="F47" s="1" t="s">
+      <c r="F48" t="s">
         <v>217</v>
       </c>
-      <c r="G47" s="1"/>
-    </row>
-    <row r="48" spans="1:7">
-      <c r="A48" t="s">
+      <c r="H48" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
+      <c r="A49" t="s">
         <v>75</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B49" t="s">
         <v>76</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C49" t="s">
         <v>148</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D49" t="s">
         <v>175</v>
       </c>
-      <c r="E48" t="s">
+      <c r="E49" t="s">
         <v>77</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="F49" t="s">
         <v>212</v>
       </c>
-      <c r="G48" s="1" t="s">
+      <c r="G49" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="49" spans="1:7" hidden="1">
-      <c r="A49" t="s">
+      <c r="H49" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" hidden="1">
+      <c r="A50" t="s">
         <v>78</v>
       </c>
-      <c r="B49" t="s">
-        <v>1</v>
-      </c>
-      <c r="E49" t="s">
-        <v>2</v>
-      </c>
-      <c r="F49" s="1"/>
-      <c r="G49" s="1"/>
-    </row>
-    <row r="50" spans="1:7">
-      <c r="A50" t="s">
+      <c r="B50" t="s">
+        <v>1</v>
+      </c>
+      <c r="E50" t="s">
+        <v>2</v>
+      </c>
+      <c r="H50" s="3"/>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" t="s">
         <v>79</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B51" t="s">
         <v>163</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C51" t="s">
         <v>150</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D51" t="s">
         <v>176</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E51" t="s">
         <v>166</v>
       </c>
-      <c r="F50" s="1" t="s">
+      <c r="F51" t="s">
         <v>236</v>
       </c>
-      <c r="G50" s="1" t="s">
+      <c r="G51" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="51" spans="1:7">
-      <c r="A51" t="s">
+      <c r="H51" s="3" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" t="s">
         <v>80</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B52" t="s">
         <v>81</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C52" t="s">
         <v>149</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D52" t="s">
         <v>159</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E52" t="s">
         <v>82</v>
       </c>
-      <c r="F51" s="1" t="s">
+      <c r="F52" t="s">
         <v>238</v>
       </c>
-      <c r="G51" s="1" t="s">
+      <c r="G52" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="52" spans="1:7">
-      <c r="A52" t="s">
+      <c r="H52" s="3" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53" t="s">
         <v>83</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B53" t="s">
         <v>84</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C53" t="s">
         <v>146</v>
       </c>
-      <c r="D52" t="s">
+      <c r="D53" t="s">
         <v>160</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E53" t="s">
         <v>13</v>
       </c>
-      <c r="F52" s="1" t="s">
+      <c r="F53" t="s">
         <v>220</v>
       </c>
-      <c r="G52" s="1" t="s">
+      <c r="G53" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="53" spans="1:7">
-      <c r="A53" t="s">
+      <c r="H53" s="3" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54" t="s">
         <v>85</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B54" t="s">
         <v>86</v>
       </c>
-      <c r="C53" t="s">
+      <c r="C54" t="s">
         <v>148</v>
       </c>
-      <c r="D53" t="s">
+      <c r="D54" t="s">
         <v>177</v>
       </c>
-      <c r="E53" t="s">
+      <c r="E54" t="s">
         <v>87</v>
       </c>
-      <c r="F53" s="1" t="s">
+      <c r="F54" t="s">
         <v>241</v>
       </c>
-      <c r="G53" s="1" t="s">
+      <c r="G54" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="54" spans="1:7" hidden="1">
-      <c r="A54" t="s">
+      <c r="H54" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" hidden="1">
+      <c r="A55" t="s">
         <v>88</v>
       </c>
-      <c r="B54" t="s">
-        <v>1</v>
-      </c>
-      <c r="E54" t="s">
-        <v>2</v>
-      </c>
-      <c r="F54" s="1"/>
-      <c r="G54" s="1"/>
-    </row>
-    <row r="55" spans="1:7" hidden="1">
-      <c r="A55" t="s">
+      <c r="B55" t="s">
+        <v>1</v>
+      </c>
+      <c r="E55" t="s">
+        <v>2</v>
+      </c>
+      <c r="H55" s="3"/>
+    </row>
+    <row r="56" spans="1:8" hidden="1">
+      <c r="A56" t="s">
         <v>89</v>
       </c>
-      <c r="B55" t="s">
-        <v>1</v>
-      </c>
-      <c r="E55" t="s">
+      <c r="B56" t="s">
+        <v>1</v>
+      </c>
+      <c r="E56" t="s">
         <v>13</v>
       </c>
-      <c r="F55" s="1"/>
-      <c r="G55" s="1"/>
-    </row>
-    <row r="56" spans="1:7">
-      <c r="A56" t="s">
+      <c r="H56" s="3"/>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57" t="s">
         <v>90</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B57" t="s">
         <v>167</v>
       </c>
-      <c r="C56" t="s">
+      <c r="C57" t="s">
         <v>150</v>
       </c>
-      <c r="D56" t="s">
+      <c r="D57" t="s">
         <v>178</v>
       </c>
-      <c r="E56" t="s">
-        <v>2</v>
-      </c>
-      <c r="F56" s="1" t="s">
+      <c r="E57" t="s">
+        <v>2</v>
+      </c>
+      <c r="F57" t="s">
         <v>221</v>
       </c>
-      <c r="G56" s="1" t="s">
+      <c r="G57" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="57" spans="1:7">
-      <c r="A57" t="s">
+      <c r="H57" s="3" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
+      <c r="A58" t="s">
         <v>91</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B58" t="s">
         <v>92</v>
       </c>
-      <c r="C57" t="s">
+      <c r="C58" t="s">
         <v>147</v>
       </c>
-      <c r="D57" t="s">
+      <c r="D58" t="s">
         <v>168</v>
       </c>
-      <c r="E57" t="s">
+      <c r="E58" t="s">
         <v>93</v>
       </c>
-      <c r="F57" s="1" t="s">
+      <c r="F58" t="s">
         <v>245</v>
       </c>
-      <c r="G57" s="1" t="s">
+      <c r="G58" t="s">
         <v>244</v>
       </c>
-    </row>
-    <row r="58" spans="1:7" hidden="1">
-      <c r="A58" t="s">
+      <c r="H58" s="3" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" hidden="1">
+      <c r="A59" t="s">
         <v>94</v>
       </c>
-      <c r="B58" t="s">
-        <v>1</v>
-      </c>
-      <c r="E58" t="s">
-        <v>2</v>
-      </c>
-      <c r="F58" s="1"/>
-      <c r="G58" s="1"/>
-    </row>
-    <row r="59" spans="1:7" hidden="1">
-      <c r="A59" t="s">
+      <c r="B59" t="s">
+        <v>1</v>
+      </c>
+      <c r="E59" t="s">
+        <v>2</v>
+      </c>
+      <c r="H59" s="3"/>
+    </row>
+    <row r="60" spans="1:8" hidden="1">
+      <c r="A60" t="s">
         <v>95</v>
       </c>
-      <c r="B59" t="s">
-        <v>1</v>
-      </c>
-      <c r="E59" t="s">
-        <v>2</v>
-      </c>
-      <c r="F59" s="1"/>
-      <c r="G59" s="1"/>
-    </row>
-    <row r="60" spans="1:7">
-      <c r="A60" t="s">
+      <c r="B60" t="s">
+        <v>1</v>
+      </c>
+      <c r="E60" t="s">
+        <v>2</v>
+      </c>
+      <c r="H60" s="3"/>
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61" t="s">
         <v>96</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B61" t="s">
         <v>97</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C61" t="s">
         <v>148</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D61" t="s">
         <v>161</v>
       </c>
-      <c r="E60" t="s">
+      <c r="E61" t="s">
         <v>98</v>
       </c>
-      <c r="F60" s="1" t="s">
+      <c r="F61" t="s">
         <v>217</v>
       </c>
-      <c r="G60" s="1"/>
-    </row>
-    <row r="61" spans="1:7" hidden="1">
-      <c r="A61" t="s">
+      <c r="H61" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" hidden="1">
+      <c r="A62" t="s">
         <v>99</v>
       </c>
-      <c r="B61" t="s">
-        <v>1</v>
-      </c>
-      <c r="E61" t="s">
-        <v>2</v>
-      </c>
-      <c r="F61" s="1"/>
-      <c r="G61" s="1"/>
-    </row>
-    <row r="62" spans="1:7" hidden="1">
-      <c r="A62" t="s">
+      <c r="B62" t="s">
+        <v>1</v>
+      </c>
+      <c r="E62" t="s">
+        <v>2</v>
+      </c>
+      <c r="H62" s="3"/>
+    </row>
+    <row r="63" spans="1:8" hidden="1">
+      <c r="A63" t="s">
         <v>100</v>
       </c>
-      <c r="B62" t="s">
-        <v>1</v>
-      </c>
-      <c r="E62" t="s">
-        <v>2</v>
-      </c>
-      <c r="F62" s="1"/>
-      <c r="G62" s="1"/>
-    </row>
-    <row r="63" spans="1:7" hidden="1">
-      <c r="A63" t="s">
+      <c r="B63" t="s">
+        <v>1</v>
+      </c>
+      <c r="E63" t="s">
+        <v>2</v>
+      </c>
+      <c r="H63" s="3"/>
+    </row>
+    <row r="64" spans="1:8" hidden="1">
+      <c r="A64" t="s">
         <v>101</v>
       </c>
-      <c r="B63" t="s">
-        <v>1</v>
-      </c>
-      <c r="E63" t="s">
-        <v>2</v>
-      </c>
-      <c r="F63" s="1"/>
-      <c r="G63" s="1"/>
-    </row>
-    <row r="64" spans="1:7" hidden="1">
-      <c r="A64" t="s">
+      <c r="B64" t="s">
+        <v>1</v>
+      </c>
+      <c r="E64" t="s">
+        <v>2</v>
+      </c>
+      <c r="H64" s="3"/>
+    </row>
+    <row r="65" spans="1:8" hidden="1">
+      <c r="A65" t="s">
         <v>102</v>
       </c>
-      <c r="B64" t="s">
-        <v>1</v>
-      </c>
-      <c r="E64" t="s">
-        <v>2</v>
-      </c>
-      <c r="F64" s="1"/>
-      <c r="G64" s="1"/>
-    </row>
-    <row r="65" spans="1:7" ht="45">
-      <c r="A65" t="s">
+      <c r="B65" t="s">
+        <v>1</v>
+      </c>
+      <c r="E65" t="s">
+        <v>2</v>
+      </c>
+      <c r="H65" s="3"/>
+    </row>
+    <row r="66" spans="1:8" ht="28.8">
+      <c r="A66" t="s">
         <v>103</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B66" t="s">
         <v>179</v>
       </c>
-      <c r="C65" t="s">
+      <c r="C66" t="s">
         <v>150</v>
       </c>
-      <c r="D65" t="s">
+      <c r="D66" t="s">
         <v>180</v>
       </c>
-      <c r="E65" t="s">
+      <c r="E66" t="s">
         <v>181</v>
       </c>
-      <c r="F65" s="1" t="s">
+      <c r="F66" t="s">
         <v>246</v>
       </c>
-      <c r="G65" s="3" t="s">
+      <c r="G66" s="2" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="66" spans="1:7" hidden="1">
-      <c r="A66" t="s">
+      <c r="H66" s="4" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" hidden="1">
+      <c r="A67" t="s">
         <v>104</v>
       </c>
-      <c r="B66" t="s">
-        <v>1</v>
-      </c>
-      <c r="E66" t="s">
-        <v>2</v>
-      </c>
-      <c r="F66" s="1"/>
-      <c r="G66" s="1"/>
-    </row>
-    <row r="67" spans="1:7" hidden="1">
-      <c r="A67" t="s">
+      <c r="B67" t="s">
+        <v>1</v>
+      </c>
+      <c r="E67" t="s">
+        <v>2</v>
+      </c>
+      <c r="H67" s="3"/>
+    </row>
+    <row r="68" spans="1:8" hidden="1">
+      <c r="A68" t="s">
         <v>105</v>
       </c>
-      <c r="B67" t="s">
-        <v>1</v>
-      </c>
-      <c r="E67" t="s">
-        <v>2</v>
-      </c>
-      <c r="F67" s="1"/>
-      <c r="G67" s="1"/>
-    </row>
-    <row r="68" spans="1:7" hidden="1">
-      <c r="A68" t="s">
+      <c r="B68" t="s">
+        <v>1</v>
+      </c>
+      <c r="E68" t="s">
+        <v>2</v>
+      </c>
+      <c r="H68" s="3"/>
+    </row>
+    <row r="69" spans="1:8" hidden="1">
+      <c r="A69" t="s">
         <v>106</v>
       </c>
-      <c r="B68" t="s">
-        <v>1</v>
-      </c>
-      <c r="E68" t="s">
-        <v>2</v>
-      </c>
-      <c r="F68" s="1"/>
-      <c r="G68" s="1"/>
-    </row>
-    <row r="69" spans="1:7" hidden="1">
-      <c r="A69" t="s">
+      <c r="B69" t="s">
+        <v>1</v>
+      </c>
+      <c r="E69" t="s">
+        <v>2</v>
+      </c>
+      <c r="H69" s="3"/>
+    </row>
+    <row r="70" spans="1:8" hidden="1">
+      <c r="A70" t="s">
         <v>107</v>
       </c>
-      <c r="B69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E69" t="s">
-        <v>2</v>
-      </c>
-      <c r="F69" s="1"/>
-      <c r="G69" s="1"/>
-    </row>
-    <row r="70" spans="1:7" hidden="1">
-      <c r="A70" t="s">
+      <c r="B70" t="s">
+        <v>1</v>
+      </c>
+      <c r="E70" t="s">
+        <v>2</v>
+      </c>
+      <c r="H70" s="3"/>
+    </row>
+    <row r="71" spans="1:8" hidden="1">
+      <c r="A71" t="s">
         <v>108</v>
       </c>
-      <c r="B70" t="s">
-        <v>1</v>
-      </c>
-      <c r="E70" t="s">
-        <v>2</v>
-      </c>
-      <c r="F70" s="1"/>
-      <c r="G70" s="1"/>
-    </row>
-    <row r="71" spans="1:7" hidden="1">
-      <c r="A71" t="s">
+      <c r="B71" t="s">
+        <v>1</v>
+      </c>
+      <c r="E71" t="s">
+        <v>2</v>
+      </c>
+      <c r="H71" s="3"/>
+    </row>
+    <row r="72" spans="1:8" hidden="1">
+      <c r="A72" t="s">
         <v>109</v>
       </c>
-      <c r="B71" t="s">
-        <v>1</v>
-      </c>
-      <c r="E71" t="s">
-        <v>2</v>
-      </c>
-      <c r="F71" s="1"/>
-      <c r="G71" s="1"/>
-    </row>
-    <row r="72" spans="1:7" hidden="1">
-      <c r="A72" t="s">
+      <c r="B72" t="s">
+        <v>1</v>
+      </c>
+      <c r="E72" t="s">
+        <v>2</v>
+      </c>
+      <c r="H72" s="3"/>
+    </row>
+    <row r="73" spans="1:8" hidden="1">
+      <c r="A73" t="s">
         <v>110</v>
       </c>
-      <c r="B72" t="s">
-        <v>1</v>
-      </c>
-      <c r="E72" t="s">
-        <v>2</v>
-      </c>
-      <c r="F72" s="1"/>
-      <c r="G72" s="1"/>
-    </row>
-    <row r="73" spans="1:7" hidden="1">
-      <c r="A73" t="s">
+      <c r="B73" t="s">
+        <v>1</v>
+      </c>
+      <c r="E73" t="s">
+        <v>2</v>
+      </c>
+      <c r="H73" s="3"/>
+    </row>
+    <row r="74" spans="1:8" hidden="1">
+      <c r="A74" t="s">
         <v>111</v>
       </c>
-      <c r="B73" t="s">
-        <v>1</v>
-      </c>
-      <c r="E73" t="s">
-        <v>2</v>
-      </c>
-      <c r="F73" s="1"/>
-      <c r="G73" s="1"/>
-    </row>
-    <row r="74" spans="1:7" ht="30">
-      <c r="A74" t="s">
+      <c r="B74" t="s">
+        <v>1</v>
+      </c>
+      <c r="E74" t="s">
+        <v>2</v>
+      </c>
+      <c r="H74" s="3"/>
+    </row>
+    <row r="75" spans="1:8" ht="28.8">
+      <c r="A75" t="s">
         <v>112</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B75" t="s">
         <v>113</v>
       </c>
-      <c r="C74" t="s">
+      <c r="C75" t="s">
         <v>148</v>
       </c>
-      <c r="D74" t="s">
+      <c r="D75" t="s">
         <v>188</v>
       </c>
-      <c r="E74" t="s">
+      <c r="E75" t="s">
         <v>114</v>
       </c>
-      <c r="F74" s="1" t="s">
+      <c r="F75" t="s">
         <v>249</v>
       </c>
-      <c r="G74" s="3" t="s">
+      <c r="G75" s="2" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="75" spans="1:7" hidden="1">
-      <c r="A75" t="s">
+      <c r="H75" s="4" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" hidden="1">
+      <c r="A76" t="s">
         <v>115</v>
       </c>
-      <c r="B75" t="s">
-        <v>1</v>
-      </c>
-      <c r="E75" t="s">
-        <v>2</v>
-      </c>
-      <c r="F75" s="1"/>
-      <c r="G75" s="1"/>
-    </row>
-    <row r="76" spans="1:7">
-      <c r="A76" t="s">
+      <c r="B76" t="s">
+        <v>1</v>
+      </c>
+      <c r="E76" t="s">
+        <v>2</v>
+      </c>
+      <c r="H76" s="3"/>
+    </row>
+    <row r="77" spans="1:8">
+      <c r="A77" t="s">
         <v>116</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B77" t="s">
         <v>117</v>
       </c>
-      <c r="C76" t="s">
+      <c r="C77" t="s">
         <v>148</v>
       </c>
-      <c r="D76" t="s">
+      <c r="D77" t="s">
         <v>189</v>
       </c>
-      <c r="E76" t="s">
+      <c r="E77" t="s">
         <v>118</v>
       </c>
-      <c r="F76" s="1" t="s">
+      <c r="F77" t="s">
         <v>250</v>
       </c>
-      <c r="G76" s="1" t="s">
+      <c r="G77" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="77" spans="1:7" hidden="1">
-      <c r="A77" t="s">
+      <c r="H77" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" hidden="1">
+      <c r="A78" t="s">
         <v>119</v>
       </c>
-      <c r="B77" t="s">
-        <v>1</v>
-      </c>
-      <c r="E77" t="s">
-        <v>2</v>
-      </c>
-      <c r="F77" s="1"/>
-      <c r="G77" s="1"/>
-    </row>
-    <row r="78" spans="1:7" hidden="1">
-      <c r="A78" t="s">
+      <c r="B78" t="s">
+        <v>1</v>
+      </c>
+      <c r="E78" t="s">
+        <v>2</v>
+      </c>
+      <c r="H78" s="3"/>
+    </row>
+    <row r="79" spans="1:8" hidden="1">
+      <c r="A79" t="s">
         <v>120</v>
       </c>
-      <c r="B78" t="s">
-        <v>1</v>
-      </c>
-      <c r="E78" t="s">
-        <v>2</v>
-      </c>
-      <c r="F78" s="1"/>
-      <c r="G78" s="1"/>
-    </row>
-    <row r="79" spans="1:7" hidden="1">
-      <c r="A79" t="s">
+      <c r="B79" t="s">
+        <v>1</v>
+      </c>
+      <c r="E79" t="s">
+        <v>2</v>
+      </c>
+      <c r="H79" s="3"/>
+    </row>
+    <row r="80" spans="1:8" hidden="1">
+      <c r="A80" t="s">
         <v>121</v>
       </c>
-      <c r="B79" t="s">
-        <v>1</v>
-      </c>
-      <c r="E79" t="s">
-        <v>2</v>
-      </c>
-      <c r="F79" s="1"/>
-      <c r="G79" s="1"/>
-    </row>
-    <row r="80" spans="1:7" hidden="1">
-      <c r="A80" t="s">
+      <c r="B80" t="s">
+        <v>1</v>
+      </c>
+      <c r="E80" t="s">
+        <v>2</v>
+      </c>
+      <c r="H80" s="3"/>
+    </row>
+    <row r="81" spans="1:8" hidden="1">
+      <c r="A81" t="s">
         <v>122</v>
       </c>
-      <c r="B80" t="s">
-        <v>1</v>
-      </c>
-      <c r="E80" t="s">
-        <v>2</v>
-      </c>
-      <c r="F80" s="1"/>
-      <c r="G80" s="1"/>
-    </row>
-    <row r="81" spans="1:7" hidden="1">
-      <c r="A81" t="s">
+      <c r="B81" t="s">
+        <v>1</v>
+      </c>
+      <c r="E81" t="s">
+        <v>2</v>
+      </c>
+      <c r="H81" s="3"/>
+    </row>
+    <row r="82" spans="1:8" hidden="1">
+      <c r="A82" t="s">
         <v>123</v>
       </c>
-      <c r="B81" t="s">
-        <v>1</v>
-      </c>
-      <c r="E81" t="s">
-        <v>2</v>
-      </c>
-      <c r="F81" s="1"/>
-      <c r="G81" s="1"/>
-    </row>
-    <row r="82" spans="1:7">
-      <c r="A82" t="s">
+      <c r="B82" t="s">
+        <v>1</v>
+      </c>
+      <c r="E82" t="s">
+        <v>2</v>
+      </c>
+      <c r="H82" s="3"/>
+    </row>
+    <row r="83" spans="1:8">
+      <c r="A83" t="s">
         <v>124</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B83" t="s">
         <v>125</v>
-      </c>
-      <c r="C82" t="s">
-        <v>146</v>
-      </c>
-      <c r="D82" t="s">
-        <v>190</v>
-      </c>
-      <c r="E82" t="s">
-        <v>13</v>
-      </c>
-      <c r="F82" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="G82" s="1" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7">
-      <c r="A83" t="s">
-        <v>126</v>
-      </c>
-      <c r="B83" t="s">
-        <v>127</v>
       </c>
       <c r="C83" t="s">
         <v>146</v>
       </c>
       <c r="D83" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="E83" t="s">
         <v>13</v>
       </c>
-      <c r="F83" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="G83" s="1" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7">
+      <c r="F83" t="s">
+        <v>222</v>
+      </c>
+      <c r="G83" t="s">
+        <v>252</v>
+      </c>
+      <c r="H83" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8">
       <c r="A84" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B84" t="s">
-        <v>182</v>
+        <v>127</v>
       </c>
       <c r="C84" t="s">
         <v>146</v>
       </c>
       <c r="D84" t="s">
+        <v>184</v>
+      </c>
+      <c r="E84" t="s">
+        <v>13</v>
+      </c>
+      <c r="F84" t="s">
+        <v>223</v>
+      </c>
+      <c r="G84" t="s">
+        <v>253</v>
+      </c>
+      <c r="H84" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8">
+      <c r="A85" t="s">
+        <v>128</v>
+      </c>
+      <c r="B85" t="s">
+        <v>182</v>
+      </c>
+      <c r="C85" t="s">
+        <v>146</v>
+      </c>
+      <c r="D85" t="s">
         <v>183</v>
       </c>
-      <c r="E84" t="s">
-        <v>2</v>
-      </c>
-      <c r="F84" s="1" t="s">
+      <c r="E85" t="s">
+        <v>2</v>
+      </c>
+      <c r="F85" t="s">
         <v>224</v>
       </c>
-      <c r="G84" s="1" t="s">
+      <c r="G85" t="s">
         <v>256</v>
       </c>
-    </row>
-    <row r="85" spans="1:7" hidden="1">
-      <c r="A85" t="s">
+      <c r="H85" s="3" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" hidden="1">
+      <c r="A86" t="s">
         <v>129</v>
       </c>
-      <c r="B85" t="s">
-        <v>1</v>
-      </c>
-      <c r="E85" t="s">
-        <v>2</v>
-      </c>
-      <c r="F85" s="1"/>
-      <c r="G85" s="1"/>
-    </row>
-    <row r="86" spans="1:7" hidden="1">
-      <c r="A86" t="s">
+      <c r="B86" t="s">
+        <v>1</v>
+      </c>
+      <c r="E86" t="s">
+        <v>2</v>
+      </c>
+      <c r="H86" s="3"/>
+    </row>
+    <row r="87" spans="1:8" hidden="1">
+      <c r="A87" t="s">
         <v>130</v>
       </c>
-      <c r="B86" t="s">
-        <v>1</v>
-      </c>
-      <c r="E86" t="s">
-        <v>2</v>
-      </c>
-      <c r="F86" s="1"/>
-      <c r="G86" s="1"/>
-    </row>
-    <row r="87" spans="1:7" hidden="1">
-      <c r="A87" t="s">
+      <c r="B87" t="s">
+        <v>1</v>
+      </c>
+      <c r="E87" t="s">
+        <v>2</v>
+      </c>
+      <c r="H87" s="3"/>
+    </row>
+    <row r="88" spans="1:8" hidden="1">
+      <c r="A88" t="s">
         <v>131</v>
       </c>
-      <c r="B87" t="s">
-        <v>1</v>
-      </c>
-      <c r="E87" t="s">
-        <v>2</v>
-      </c>
-      <c r="F87" s="1"/>
-      <c r="G87" s="1"/>
-    </row>
-    <row r="88" spans="1:7" hidden="1">
-      <c r="A88" t="s">
+      <c r="B88" t="s">
+        <v>1</v>
+      </c>
+      <c r="E88" t="s">
+        <v>2</v>
+      </c>
+      <c r="H88" s="3"/>
+    </row>
+    <row r="89" spans="1:8" hidden="1">
+      <c r="A89" t="s">
         <v>132</v>
       </c>
-      <c r="B88" t="s">
-        <v>1</v>
-      </c>
-      <c r="E88" t="s">
-        <v>2</v>
-      </c>
-      <c r="F88" s="1"/>
-      <c r="G88" s="1"/>
-    </row>
-    <row r="89" spans="1:7" hidden="1">
-      <c r="A89" t="s">
+      <c r="B89" t="s">
+        <v>1</v>
+      </c>
+      <c r="E89" t="s">
+        <v>2</v>
+      </c>
+      <c r="H89" s="3"/>
+    </row>
+    <row r="90" spans="1:8" hidden="1">
+      <c r="A90" t="s">
         <v>133</v>
       </c>
-      <c r="B89" t="s">
-        <v>1</v>
-      </c>
-      <c r="E89" t="s">
-        <v>2</v>
-      </c>
-      <c r="F89" s="1"/>
-      <c r="G89" s="1"/>
-    </row>
-    <row r="90" spans="1:7" hidden="1">
-      <c r="A90" t="s">
+      <c r="B90" t="s">
+        <v>1</v>
+      </c>
+      <c r="E90" t="s">
+        <v>2</v>
+      </c>
+      <c r="H90" s="3"/>
+    </row>
+    <row r="91" spans="1:8" hidden="1">
+      <c r="A91" t="s">
         <v>134</v>
       </c>
-      <c r="B90" t="s">
-        <v>1</v>
-      </c>
-      <c r="E90" t="s">
-        <v>2</v>
-      </c>
-      <c r="F90" s="1"/>
-      <c r="G90" s="1"/>
-    </row>
-    <row r="91" spans="1:7" hidden="1">
-      <c r="A91" t="s">
+      <c r="B91" t="s">
+        <v>1</v>
+      </c>
+      <c r="E91" t="s">
+        <v>2</v>
+      </c>
+      <c r="H91" s="3"/>
+    </row>
+    <row r="92" spans="1:8" hidden="1">
+      <c r="A92" t="s">
         <v>135</v>
       </c>
-      <c r="B91" t="s">
-        <v>1</v>
-      </c>
-      <c r="E91" t="s">
-        <v>2</v>
-      </c>
-      <c r="F91" s="1"/>
-      <c r="G91" s="1"/>
-    </row>
-    <row r="92" spans="1:7" hidden="1">
-      <c r="A92" t="s">
+      <c r="B92" t="s">
+        <v>1</v>
+      </c>
+      <c r="E92" t="s">
+        <v>2</v>
+      </c>
+      <c r="H92" s="3"/>
+    </row>
+    <row r="93" spans="1:8" hidden="1">
+      <c r="A93" t="s">
         <v>136</v>
       </c>
-      <c r="B92" t="s">
-        <v>1</v>
-      </c>
-      <c r="E92" t="s">
-        <v>2</v>
-      </c>
-      <c r="F92" s="1"/>
-      <c r="G92" s="1"/>
-    </row>
-    <row r="93" spans="1:7" hidden="1">
-      <c r="A93" t="s">
+      <c r="B93" t="s">
+        <v>1</v>
+      </c>
+      <c r="E93" t="s">
+        <v>2</v>
+      </c>
+      <c r="H93" s="3"/>
+    </row>
+    <row r="94" spans="1:8" hidden="1">
+      <c r="A94" t="s">
         <v>137</v>
       </c>
-      <c r="B93" t="s">
-        <v>1</v>
-      </c>
-      <c r="E93" t="s">
-        <v>2</v>
-      </c>
-      <c r="F93" s="1"/>
-      <c r="G93" s="1"/>
-    </row>
-    <row r="94" spans="1:7" ht="60">
-      <c r="A94" t="s">
+      <c r="B94" t="s">
+        <v>1</v>
+      </c>
+      <c r="E94" t="s">
+        <v>2</v>
+      </c>
+      <c r="H94" s="3"/>
+    </row>
+    <row r="95" spans="1:8" ht="57.6">
+      <c r="A95" t="s">
         <v>138</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B95" t="s">
         <v>185</v>
       </c>
-      <c r="C94" t="s">
+      <c r="C95" t="s">
         <v>150</v>
       </c>
-      <c r="D94" t="s">
+      <c r="D95" t="s">
         <v>187</v>
       </c>
-      <c r="E94" t="s">
+      <c r="E95" t="s">
         <v>186</v>
       </c>
-      <c r="F94" s="1" t="s">
+      <c r="F95" t="s">
         <v>254</v>
       </c>
-      <c r="G94" s="3" t="s">
+      <c r="G95" s="2" t="s">
         <v>255</v>
+      </c>
+      <c r="H95" s="4" t="s">
+        <v>259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>